<commit_message>
chore: actualizar datos y reporte web
</commit_message>
<xml_diff>
--- a/data-coyuntura.xlsx
+++ b/data-coyuntura.xlsx
@@ -14329,7 +14329,9 @@
       </c>
       <c r="D314"/>
       <c r="E314"/>
-      <c r="F314"/>
+      <c r="F314" t="n">
+        <v>129.96287646414</v>
+      </c>
       <c r="G314" t="n">
         <v>4.89226213151006</v>
       </c>
@@ -14346,8 +14348,12 @@
       <c r="L314"/>
       <c r="M314"/>
       <c r="N314"/>
-      <c r="O314"/>
-      <c r="P314"/>
+      <c r="O314" t="n">
+        <v>3.48006152430886</v>
+      </c>
+      <c r="P314" t="n">
+        <v>-2.09683553036542</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -45419,85 +45425,85 @@
         <v>46054</v>
       </c>
       <c r="B363" t="n">
-        <v>57973.2475572784</v>
+        <v>57549.7794852784</v>
       </c>
       <c r="C363" t="n">
-        <v>6666.545969</v>
+        <v>6622.99956</v>
       </c>
       <c r="D363" t="n">
-        <v>145474.863034673</v>
+        <v>145130.179789673</v>
       </c>
       <c r="E363" t="n">
-        <v>113485.59868</v>
+        <v>113137.980913</v>
       </c>
       <c r="F363" t="n">
-        <v>169155.843628</v>
+        <v>169773.175196</v>
       </c>
       <c r="G363" t="n">
-        <v>371614.953204897</v>
+        <v>370377.506594897</v>
       </c>
       <c r="H363" t="n">
-        <v>105893.576773</v>
+        <v>104869.268935</v>
       </c>
       <c r="I363" t="n">
-        <v>47970.8255175668</v>
+        <v>47973.2077435668</v>
       </c>
       <c r="J363" t="n">
-        <v>113084.754742</v>
+        <v>112965.661497</v>
       </c>
       <c r="K363" t="n">
-        <v>462183.210062015</v>
+        <v>462467.834094015</v>
       </c>
       <c r="L363" t="n">
-        <v>47851.46972</v>
+        <v>47820.907982</v>
       </c>
       <c r="M363" t="n">
-        <v>82868.53079</v>
+        <v>82962.31583</v>
       </c>
       <c r="N363" t="n">
-        <v>683670.093517629</v>
+        <v>683333.497783629</v>
       </c>
       <c r="O363" t="n">
-        <v>125530.159585</v>
+        <v>125281.41503</v>
       </c>
       <c r="P363" t="n">
-        <v>558139.933932629</v>
+        <v>558052.082753629</v>
       </c>
       <c r="Q363" t="n">
-        <v>102571.458437454</v>
+        <v>103106.758983454</v>
       </c>
       <c r="R363" t="n">
-        <v>2618569.74193914</v>
+        <v>2619744.14868014</v>
       </c>
       <c r="S363" t="n">
-        <v>575565.323212</v>
+        <v>571680.423491</v>
       </c>
       <c r="T363" t="n">
-        <v>3194135.06515114</v>
+        <v>3191424.57217114</v>
       </c>
       <c r="U363" t="n">
-        <v>0.497260430405122</v>
+        <v>0.542332615503427</v>
       </c>
       <c r="V363" t="n">
-        <v>7.14225576759655</v>
+        <v>7.19030817781274</v>
       </c>
       <c r="W363" t="n">
-        <v>-2.47968756849192</v>
+        <v>-3.13792151567058</v>
       </c>
       <c r="X363" t="n">
-        <v>6.48263289180817</v>
+        <v>5.76390586964468</v>
       </c>
       <c r="Y363" t="n">
-        <v>-0.0525201010615706</v>
+        <v>-0.137333966821473</v>
       </c>
       <c r="Z363" t="n">
-        <v>7.02279245580524</v>
+        <v>6.9319745906447</v>
       </c>
       <c r="AA363" t="n">
-        <v>0.81980557757511</v>
+        <v>0.820869830834798</v>
       </c>
       <c r="AB363" t="n">
-        <v>0.180194422424891</v>
+        <v>0.179130169165202</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
se agrego la función de los datos de tarjetas de créditos
</commit_message>
<xml_diff>
--- a/data-coyuntura.xlsx
+++ b/data-coyuntura.xlsx
@@ -9,12 +9,13 @@
     <sheet name="índices" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="préstamos" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="IPC" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="sipen" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="369">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="372">
   <si>
     <t xml:space="preserve">fecha</t>
   </si>
@@ -1122,6 +1123,15 @@
   <si>
     <t xml:space="preserve">127.6391</t>
   </si>
+  <si>
+    <t xml:space="preserve">mes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">salario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cotizantes</t>
+  </si>
 </sst>
 </file>
 
@@ -58827,4 +58837,3047 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>369</v>
+      </c>
+      <c r="B1" t="s">
+        <v>370</v>
+      </c>
+      <c r="C1" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n">
+        <v>37833</v>
+      </c>
+      <c r="B2" t="n">
+        <v>7088.2099609375</v>
+      </c>
+      <c r="C2"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n">
+        <v>37864</v>
+      </c>
+      <c r="B3" t="n">
+        <v>6637.5498046875</v>
+      </c>
+      <c r="C3"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="n">
+        <v>37894</v>
+      </c>
+      <c r="B4" t="n">
+        <v>6983.14990234375</v>
+      </c>
+      <c r="C4" t="n">
+        <v>570119</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="n">
+        <v>37925</v>
+      </c>
+      <c r="B5" t="n">
+        <v>7067.77978515625</v>
+      </c>
+      <c r="C5" t="n">
+        <v>571062</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="n">
+        <v>37955</v>
+      </c>
+      <c r="B6" t="n">
+        <v>7229.75</v>
+      </c>
+      <c r="C6" t="n">
+        <v>573216</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="n">
+        <v>37986</v>
+      </c>
+      <c r="B7" t="n">
+        <v>7407.06005859375</v>
+      </c>
+      <c r="C7" t="n">
+        <v>576869</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n">
+        <v>38017</v>
+      </c>
+      <c r="B8" t="n">
+        <v>7641.8798828125</v>
+      </c>
+      <c r="C8" t="n">
+        <v>510977</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n">
+        <v>38046</v>
+      </c>
+      <c r="B9" t="n">
+        <v>7657.759765625</v>
+      </c>
+      <c r="C9" t="n">
+        <v>577717</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="n">
+        <v>38077</v>
+      </c>
+      <c r="B10" t="n">
+        <v>7944.47998046875</v>
+      </c>
+      <c r="C10" t="n">
+        <v>589862</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="n">
+        <v>38107</v>
+      </c>
+      <c r="B11" t="n">
+        <v>7914.669921875</v>
+      </c>
+      <c r="C11" t="n">
+        <v>750512</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="n">
+        <v>38138</v>
+      </c>
+      <c r="B12" t="n">
+        <v>8174.35986328125</v>
+      </c>
+      <c r="C12" t="n">
+        <v>673738</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="n">
+        <v>38168</v>
+      </c>
+      <c r="B13" t="n">
+        <v>8083.31005859375</v>
+      </c>
+      <c r="C13" t="n">
+        <v>737226</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="n">
+        <v>38199</v>
+      </c>
+      <c r="B14" t="n">
+        <v>8223.4296875</v>
+      </c>
+      <c r="C14" t="n">
+        <v>741387</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="n">
+        <v>38230</v>
+      </c>
+      <c r="B15" t="n">
+        <v>8672.0595703125</v>
+      </c>
+      <c r="C15" t="n">
+        <v>604016</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="n">
+        <v>38260</v>
+      </c>
+      <c r="B16" t="n">
+        <v>8397.08984375</v>
+      </c>
+      <c r="C16" t="n">
+        <v>622183</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="n">
+        <v>38291</v>
+      </c>
+      <c r="B17" t="n">
+        <v>8651.76953125</v>
+      </c>
+      <c r="C17" t="n">
+        <v>624582</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="n">
+        <v>38321</v>
+      </c>
+      <c r="B18" t="n">
+        <v>8748.4296875</v>
+      </c>
+      <c r="C18" t="n">
+        <v>753666</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="n">
+        <v>38352</v>
+      </c>
+      <c r="B19" t="n">
+        <v>8956.1298828125</v>
+      </c>
+      <c r="C19" t="n">
+        <v>593286</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="n">
+        <v>38383</v>
+      </c>
+      <c r="B20" t="n">
+        <v>9309.8603515625</v>
+      </c>
+      <c r="C20" t="n">
+        <v>581267</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="n">
+        <v>38411</v>
+      </c>
+      <c r="B21" t="n">
+        <v>9817.8095703125</v>
+      </c>
+      <c r="C21" t="n">
+        <v>835032</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="n">
+        <v>38442</v>
+      </c>
+      <c r="B22" t="n">
+        <v>9696.830078125</v>
+      </c>
+      <c r="C22" t="n">
+        <v>725929</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="n">
+        <v>38472</v>
+      </c>
+      <c r="B23" t="n">
+        <v>11461.1298828125</v>
+      </c>
+      <c r="C23" t="n">
+        <v>733936</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="n">
+        <v>38503</v>
+      </c>
+      <c r="B24" t="n">
+        <v>10158.509765625</v>
+      </c>
+      <c r="C24" t="n">
+        <v>706720</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="n">
+        <v>38533</v>
+      </c>
+      <c r="B25" t="n">
+        <v>9867.830078125</v>
+      </c>
+      <c r="C25" t="n">
+        <v>720862</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="n">
+        <v>38564</v>
+      </c>
+      <c r="B26" t="n">
+        <v>10542.509765625</v>
+      </c>
+      <c r="C26" t="n">
+        <v>773186</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="n">
+        <v>38595</v>
+      </c>
+      <c r="B27" t="n">
+        <v>10274.6904296875</v>
+      </c>
+      <c r="C27" t="n">
+        <v>757575</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="n">
+        <v>38625</v>
+      </c>
+      <c r="B28" t="n">
+        <v>10369.2197265625</v>
+      </c>
+      <c r="C28" t="n">
+        <v>678912</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="n">
+        <v>38656</v>
+      </c>
+      <c r="B29" t="n">
+        <v>10308.76953125</v>
+      </c>
+      <c r="C29" t="n">
+        <v>733909</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="n">
+        <v>38686</v>
+      </c>
+      <c r="B30" t="n">
+        <v>10598.8603515625</v>
+      </c>
+      <c r="C30" t="n">
+        <v>657018</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="n">
+        <v>38717</v>
+      </c>
+      <c r="B31" t="n">
+        <v>10717.259765625</v>
+      </c>
+      <c r="C31" t="n">
+        <v>626615</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="n">
+        <v>38748</v>
+      </c>
+      <c r="B32" t="n">
+        <v>11213.490234375</v>
+      </c>
+      <c r="C32" t="n">
+        <v>555033</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="n">
+        <v>38776</v>
+      </c>
+      <c r="B33" t="n">
+        <v>10484.8701171875</v>
+      </c>
+      <c r="C33" t="n">
+        <v>637018</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="n">
+        <v>38807</v>
+      </c>
+      <c r="B34" t="n">
+        <v>10866.509765625</v>
+      </c>
+      <c r="C34" t="n">
+        <v>639878</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="n">
+        <v>38837</v>
+      </c>
+      <c r="B35" t="n">
+        <v>11217.73046875</v>
+      </c>
+      <c r="C35" t="n">
+        <v>742746</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="n">
+        <v>38868</v>
+      </c>
+      <c r="B36" t="n">
+        <v>10995.240234375</v>
+      </c>
+      <c r="C36" t="n">
+        <v>769270</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="n">
+        <v>38898</v>
+      </c>
+      <c r="B37" t="n">
+        <v>10919</v>
+      </c>
+      <c r="C37" t="n">
+        <v>761772</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="n">
+        <v>38929</v>
+      </c>
+      <c r="B38" t="n">
+        <v>11146.3701171875</v>
+      </c>
+      <c r="C38" t="n">
+        <v>763820</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="n">
+        <v>38960</v>
+      </c>
+      <c r="B39" t="n">
+        <v>11141.2001953125</v>
+      </c>
+      <c r="C39" t="n">
+        <v>772056</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="n">
+        <v>38990</v>
+      </c>
+      <c r="B40" t="n">
+        <v>11358.5703125</v>
+      </c>
+      <c r="C40" t="n">
+        <v>768990</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="n">
+        <v>39021</v>
+      </c>
+      <c r="B41" t="n">
+        <v>11298.08984375</v>
+      </c>
+      <c r="C41" t="n">
+        <v>790384</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="n">
+        <v>39051</v>
+      </c>
+      <c r="B42" t="n">
+        <v>11352.8896484375</v>
+      </c>
+      <c r="C42" t="n">
+        <v>785133</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="n">
+        <v>39082</v>
+      </c>
+      <c r="B43" t="n">
+        <v>11557.1396484375</v>
+      </c>
+      <c r="C43" t="n">
+        <v>808496</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="n">
+        <v>39113</v>
+      </c>
+      <c r="B44" t="n">
+        <v>11875.330078125</v>
+      </c>
+      <c r="C44" t="n">
+        <v>742001</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="n">
+        <v>39141</v>
+      </c>
+      <c r="B45" t="n">
+        <v>11335.23046875</v>
+      </c>
+      <c r="C45" t="n">
+        <v>790414</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="n">
+        <v>39172</v>
+      </c>
+      <c r="B46" t="n">
+        <v>11695.1201171875</v>
+      </c>
+      <c r="C46" t="n">
+        <v>821887</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="n">
+        <v>39202</v>
+      </c>
+      <c r="B47" t="n">
+        <v>11909.580078125</v>
+      </c>
+      <c r="C47" t="n">
+        <v>809789</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="n">
+        <v>39233</v>
+      </c>
+      <c r="B48" t="n">
+        <v>11926.08984375</v>
+      </c>
+      <c r="C48" t="n">
+        <v>838413</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="n">
+        <v>39263</v>
+      </c>
+      <c r="B49" t="n">
+        <v>12357.4697265625</v>
+      </c>
+      <c r="C49" t="n">
+        <v>837302</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="1" t="n">
+        <v>39294</v>
+      </c>
+      <c r="B50" t="n">
+        <v>12491.990234375</v>
+      </c>
+      <c r="C50" t="n">
+        <v>826642</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="n">
+        <v>39325</v>
+      </c>
+      <c r="B51" t="n">
+        <v>12455.3701171875</v>
+      </c>
+      <c r="C51" t="n">
+        <v>804054</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="1" t="n">
+        <v>39355</v>
+      </c>
+      <c r="B52" t="n">
+        <v>12426.830078125</v>
+      </c>
+      <c r="C52" t="n">
+        <v>833676</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="1" t="n">
+        <v>39386</v>
+      </c>
+      <c r="B53" t="n">
+        <v>12161.259765625</v>
+      </c>
+      <c r="C53" t="n">
+        <v>867962</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="1" t="n">
+        <v>39416</v>
+      </c>
+      <c r="B54" t="n">
+        <v>12078.1796875</v>
+      </c>
+      <c r="C54" t="n">
+        <v>876418</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="1" t="n">
+        <v>39447</v>
+      </c>
+      <c r="B55" t="n">
+        <v>12156.5595703125</v>
+      </c>
+      <c r="C55" t="n">
+        <v>913203</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="1" t="n">
+        <v>39478</v>
+      </c>
+      <c r="B56" t="n">
+        <v>12422.0302734375</v>
+      </c>
+      <c r="C56" t="n">
+        <v>832677</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="1" t="n">
+        <v>39507</v>
+      </c>
+      <c r="B57" t="n">
+        <v>12129.8203125</v>
+      </c>
+      <c r="C57" t="n">
+        <v>858797</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="1" t="n">
+        <v>39538</v>
+      </c>
+      <c r="B58" t="n">
+        <v>12360.25</v>
+      </c>
+      <c r="C58" t="n">
+        <v>901599</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="1" t="n">
+        <v>39568</v>
+      </c>
+      <c r="B59" t="n">
+        <v>12437.3896484375</v>
+      </c>
+      <c r="C59" t="n">
+        <v>882878</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="1" t="n">
+        <v>39599</v>
+      </c>
+      <c r="B60" t="n">
+        <v>12543.6298828125</v>
+      </c>
+      <c r="C60" t="n">
+        <v>908331</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="1" t="n">
+        <v>39629</v>
+      </c>
+      <c r="B61" t="n">
+        <v>12538.51953125</v>
+      </c>
+      <c r="C61" t="n">
+        <v>915787</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="1" t="n">
+        <v>39660</v>
+      </c>
+      <c r="B62" t="n">
+        <v>12592.73046875</v>
+      </c>
+      <c r="C62" t="n">
+        <v>928221</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="1" t="n">
+        <v>39691</v>
+      </c>
+      <c r="B63" t="n">
+        <v>12771.330078125</v>
+      </c>
+      <c r="C63" t="n">
+        <v>896435</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="1" t="n">
+        <v>39721</v>
+      </c>
+      <c r="B64" t="n">
+        <v>13222.98046875</v>
+      </c>
+      <c r="C64" t="n">
+        <v>921225</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="1" t="n">
+        <v>39752</v>
+      </c>
+      <c r="B65" t="n">
+        <v>13290.7099609375</v>
+      </c>
+      <c r="C65" t="n">
+        <v>928195</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="1" t="n">
+        <v>39782</v>
+      </c>
+      <c r="B66" t="n">
+        <v>13429.5</v>
+      </c>
+      <c r="C66" t="n">
+        <v>901909</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="1" t="n">
+        <v>39813</v>
+      </c>
+      <c r="B67" t="n">
+        <v>13418.419921875</v>
+      </c>
+      <c r="C67" t="n">
+        <v>929743</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="1" t="n">
+        <v>39844</v>
+      </c>
+      <c r="B68" t="n">
+        <v>13702.2001953125</v>
+      </c>
+      <c r="C68" t="n">
+        <v>855267</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="1" t="n">
+        <v>39872</v>
+      </c>
+      <c r="B69" t="n">
+        <v>13286.0400390625</v>
+      </c>
+      <c r="C69" t="n">
+        <v>920721</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="1" t="n">
+        <v>39903</v>
+      </c>
+      <c r="B70" t="n">
+        <v>13401.5498046875</v>
+      </c>
+      <c r="C70" t="n">
+        <v>938933</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="1" t="n">
+        <v>39933</v>
+      </c>
+      <c r="B71" t="n">
+        <v>13526.759765625</v>
+      </c>
+      <c r="C71" t="n">
+        <v>998192</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="1" t="n">
+        <v>39964</v>
+      </c>
+      <c r="B72" t="n">
+        <v>13608.16015625</v>
+      </c>
+      <c r="C72" t="n">
+        <v>1017529</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="1" t="n">
+        <v>39994</v>
+      </c>
+      <c r="B73" t="n">
+        <v>13580.3095703125</v>
+      </c>
+      <c r="C73" t="n">
+        <v>1019428</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="1" t="n">
+        <v>40025</v>
+      </c>
+      <c r="B74" t="n">
+        <v>13572.4501953125</v>
+      </c>
+      <c r="C74" t="n">
+        <v>1034463</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="1" t="n">
+        <v>40056</v>
+      </c>
+      <c r="B75" t="n">
+        <v>13634.8798828125</v>
+      </c>
+      <c r="C75" t="n">
+        <v>1076120</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="1" t="n">
+        <v>40086</v>
+      </c>
+      <c r="B76" t="n">
+        <v>13318.5</v>
+      </c>
+      <c r="C76" t="n">
+        <v>995191</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="1" t="n">
+        <v>40117</v>
+      </c>
+      <c r="B77" t="n">
+        <v>13419.5595703125</v>
+      </c>
+      <c r="C77" t="n">
+        <v>1094295</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="1" t="n">
+        <v>40147</v>
+      </c>
+      <c r="B78" t="n">
+        <v>13600.7001953125</v>
+      </c>
+      <c r="C78" t="n">
+        <v>1096297</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="1" t="n">
+        <v>40178</v>
+      </c>
+      <c r="B79" t="n">
+        <v>13525.5</v>
+      </c>
+      <c r="C79" t="n">
+        <v>1118293</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="1" t="n">
+        <v>40209</v>
+      </c>
+      <c r="B80" t="n">
+        <v>14882.5302734375</v>
+      </c>
+      <c r="C80" t="n">
+        <v>1026752</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="1" t="n">
+        <v>40237</v>
+      </c>
+      <c r="B81" t="n">
+        <v>14254.3095703125</v>
+      </c>
+      <c r="C81" t="n">
+        <v>1115426</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="1" t="n">
+        <v>40268</v>
+      </c>
+      <c r="B82" t="n">
+        <v>15364.1396484375</v>
+      </c>
+      <c r="C82" t="n">
+        <v>1148486</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="1" t="n">
+        <v>40298</v>
+      </c>
+      <c r="B83" t="n">
+        <v>14719.7001953125</v>
+      </c>
+      <c r="C83" t="n">
+        <v>1109033</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="1" t="n">
+        <v>40329</v>
+      </c>
+      <c r="B84" t="n">
+        <v>15021.6103515625</v>
+      </c>
+      <c r="C84" t="n">
+        <v>1126585</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="1" t="n">
+        <v>40359</v>
+      </c>
+      <c r="B85" t="n">
+        <v>14929.6396484375</v>
+      </c>
+      <c r="C85" t="n">
+        <v>1145754</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="1" t="n">
+        <v>40390</v>
+      </c>
+      <c r="B86" t="n">
+        <v>15079.26953125</v>
+      </c>
+      <c r="C86" t="n">
+        <v>1148113</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="1" t="n">
+        <v>40421</v>
+      </c>
+      <c r="B87" t="n">
+        <v>15291.8603515625</v>
+      </c>
+      <c r="C87" t="n">
+        <v>1144919</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="1" t="n">
+        <v>40451</v>
+      </c>
+      <c r="B88" t="n">
+        <v>15155.400390625</v>
+      </c>
+      <c r="C88" t="n">
+        <v>1145836</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="1" t="n">
+        <v>40482</v>
+      </c>
+      <c r="B89" t="n">
+        <v>15378.2802734375</v>
+      </c>
+      <c r="C89" t="n">
+        <v>1153219</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="1" t="n">
+        <v>40512</v>
+      </c>
+      <c r="B90" t="n">
+        <v>15556.33984375</v>
+      </c>
+      <c r="C90" t="n">
+        <v>1176723</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="1" t="n">
+        <v>40543</v>
+      </c>
+      <c r="B91" t="n">
+        <v>16596.25</v>
+      </c>
+      <c r="C91" t="n">
+        <v>1189601</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="1" t="n">
+        <v>40574</v>
+      </c>
+      <c r="B92" t="n">
+        <v>15588.830078125</v>
+      </c>
+      <c r="C92" t="n">
+        <v>1077595</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="1" t="n">
+        <v>40602</v>
+      </c>
+      <c r="B93" t="n">
+        <v>15002.0703125</v>
+      </c>
+      <c r="C93" t="n">
+        <v>1178397</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="1" t="n">
+        <v>40633</v>
+      </c>
+      <c r="B94" t="n">
+        <v>15710.1201171875</v>
+      </c>
+      <c r="C94" t="n">
+        <v>1212258</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="1" t="n">
+        <v>40663</v>
+      </c>
+      <c r="B95" t="n">
+        <v>15402.3203125</v>
+      </c>
+      <c r="C95" t="n">
+        <v>1178755</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="1" t="n">
+        <v>40694</v>
+      </c>
+      <c r="B96" t="n">
+        <v>15975.0703125</v>
+      </c>
+      <c r="C96" t="n">
+        <v>1197970</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="1" t="n">
+        <v>40724</v>
+      </c>
+      <c r="B97" t="n">
+        <v>15728.650390625</v>
+      </c>
+      <c r="C97" t="n">
+        <v>1220579</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="1" t="n">
+        <v>40755</v>
+      </c>
+      <c r="B98" t="n">
+        <v>15965.7998046875</v>
+      </c>
+      <c r="C98" t="n">
+        <v>1216389</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="1" t="n">
+        <v>40786</v>
+      </c>
+      <c r="B99" t="n">
+        <v>16506.669921875</v>
+      </c>
+      <c r="C99" t="n">
+        <v>1232426</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="1" t="n">
+        <v>40816</v>
+      </c>
+      <c r="B100" t="n">
+        <v>16322.650390625</v>
+      </c>
+      <c r="C100" t="n">
+        <v>1208846</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="1" t="n">
+        <v>40847</v>
+      </c>
+      <c r="B101" t="n">
+        <v>16479.380859375</v>
+      </c>
+      <c r="C101" t="n">
+        <v>1223060</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="1" t="n">
+        <v>40877</v>
+      </c>
+      <c r="B102" t="n">
+        <v>16545.009765625</v>
+      </c>
+      <c r="C102" t="n">
+        <v>1232680</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="1" t="n">
+        <v>40908</v>
+      </c>
+      <c r="B103" t="n">
+        <v>17531.41015625</v>
+      </c>
+      <c r="C103" t="n">
+        <v>1242780</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="1" t="n">
+        <v>40939</v>
+      </c>
+      <c r="B104" t="n">
+        <v>16687.779296875</v>
+      </c>
+      <c r="C104" t="n">
+        <v>1160674</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="1" t="n">
+        <v>40968</v>
+      </c>
+      <c r="B105" t="n">
+        <v>16394.810546875</v>
+      </c>
+      <c r="C105" t="n">
+        <v>1242050</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="1" t="n">
+        <v>40999</v>
+      </c>
+      <c r="B106" t="n">
+        <v>17035.400390625</v>
+      </c>
+      <c r="C106" t="n">
+        <v>1263326</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="1" t="n">
+        <v>41029</v>
+      </c>
+      <c r="B107" t="n">
+        <v>16662.970703125</v>
+      </c>
+      <c r="C107" t="n">
+        <v>1232216</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="1" t="n">
+        <v>41060</v>
+      </c>
+      <c r="B108" t="n">
+        <v>17325.439453125</v>
+      </c>
+      <c r="C108" t="n">
+        <v>1281168</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="1" t="n">
+        <v>41090</v>
+      </c>
+      <c r="B109" t="n">
+        <v>16576.4296875</v>
+      </c>
+      <c r="C109" t="n">
+        <v>1236530</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="1" t="n">
+        <v>41121</v>
+      </c>
+      <c r="B110" t="n">
+        <v>17303.890625</v>
+      </c>
+      <c r="C110" t="n">
+        <v>1279009</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="1" t="n">
+        <v>41152</v>
+      </c>
+      <c r="B111" t="n">
+        <v>16912.400390625</v>
+      </c>
+      <c r="C111" t="n">
+        <v>1260233</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="1" t="n">
+        <v>41182</v>
+      </c>
+      <c r="B112" t="n">
+        <v>17003.939453125</v>
+      </c>
+      <c r="C112" t="n">
+        <v>1240431</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="1" t="n">
+        <v>41213</v>
+      </c>
+      <c r="B113" t="n">
+        <v>17164.490234375</v>
+      </c>
+      <c r="C113" t="n">
+        <v>1287611</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="1" t="n">
+        <v>41243</v>
+      </c>
+      <c r="B114" t="n">
+        <v>17049.80078125</v>
+      </c>
+      <c r="C114" t="n">
+        <v>1273247</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="1" t="n">
+        <v>41274</v>
+      </c>
+      <c r="B115" t="n">
+        <v>17911.509765625</v>
+      </c>
+      <c r="C115" t="n">
+        <v>1291137</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="1" t="n">
+        <v>41305</v>
+      </c>
+      <c r="B116" t="n">
+        <v>17312.80078125</v>
+      </c>
+      <c r="C116" t="n">
+        <v>1241113</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="1" t="n">
+        <v>41333</v>
+      </c>
+      <c r="B117" t="n">
+        <v>16726.099609375</v>
+      </c>
+      <c r="C117" t="n">
+        <v>1284535</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="1" t="n">
+        <v>41364</v>
+      </c>
+      <c r="B118" t="n">
+        <v>17331.2890625</v>
+      </c>
+      <c r="C118" t="n">
+        <v>1316873</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="1" t="n">
+        <v>41394</v>
+      </c>
+      <c r="B119" t="n">
+        <v>17347.390625</v>
+      </c>
+      <c r="C119" t="n">
+        <v>1304070</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="1" t="n">
+        <v>41425</v>
+      </c>
+      <c r="B120" t="n">
+        <v>17789.939453125</v>
+      </c>
+      <c r="C120" t="n">
+        <v>1345058</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="1" t="n">
+        <v>41455</v>
+      </c>
+      <c r="B121" t="n">
+        <v>17510.73046875</v>
+      </c>
+      <c r="C121" t="n">
+        <v>1333316</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="1" t="n">
+        <v>41486</v>
+      </c>
+      <c r="B122" t="n">
+        <v>18007.08984375</v>
+      </c>
+      <c r="C122" t="n">
+        <v>1349327</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="1" t="n">
+        <v>41517</v>
+      </c>
+      <c r="B123" t="n">
+        <v>18175.720703125</v>
+      </c>
+      <c r="C123" t="n">
+        <v>1336030</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="1" t="n">
+        <v>41547</v>
+      </c>
+      <c r="B124" t="n">
+        <v>18219.75</v>
+      </c>
+      <c r="C124" t="n">
+        <v>1335886</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="1" t="n">
+        <v>41578</v>
+      </c>
+      <c r="B125" t="n">
+        <v>18393.08984375</v>
+      </c>
+      <c r="C125" t="n">
+        <v>1366703</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="1" t="n">
+        <v>41608</v>
+      </c>
+      <c r="B126" t="n">
+        <v>18212.75</v>
+      </c>
+      <c r="C126" t="n">
+        <v>1338335</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="1" t="n">
+        <v>41639</v>
+      </c>
+      <c r="B127" t="n">
+        <v>19197.720703125</v>
+      </c>
+      <c r="C127" t="n">
+        <v>1376966</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="1" t="n">
+        <v>41670</v>
+      </c>
+      <c r="B128" t="n">
+        <v>18608.91015625</v>
+      </c>
+      <c r="C128" t="n">
+        <v>1324202</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="1" t="n">
+        <v>41698</v>
+      </c>
+      <c r="B129" t="n">
+        <v>18234.91015625</v>
+      </c>
+      <c r="C129" t="n">
+        <v>1363785</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="1" t="n">
+        <v>41729</v>
+      </c>
+      <c r="B130" t="n">
+        <v>18693.470703125</v>
+      </c>
+      <c r="C130" t="n">
+        <v>1406908</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="1" t="n">
+        <v>41759</v>
+      </c>
+      <c r="B131" t="n">
+        <v>18480.0703125</v>
+      </c>
+      <c r="C131" t="n">
+        <v>1414140</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="1" t="n">
+        <v>41790</v>
+      </c>
+      <c r="B132" t="n">
+        <v>18618.80078125</v>
+      </c>
+      <c r="C132" t="n">
+        <v>1417833</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="1" t="n">
+        <v>41820</v>
+      </c>
+      <c r="B133" t="n">
+        <v>19004.880859375</v>
+      </c>
+      <c r="C133" t="n">
+        <v>1429452</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="1" t="n">
+        <v>41851</v>
+      </c>
+      <c r="B134" t="n">
+        <v>18900.359375</v>
+      </c>
+      <c r="C134" t="n">
+        <v>1449141</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="1" t="n">
+        <v>41882</v>
+      </c>
+      <c r="B135" t="n">
+        <v>18828.599609375</v>
+      </c>
+      <c r="C135" t="n">
+        <v>1420010</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="1" t="n">
+        <v>41912</v>
+      </c>
+      <c r="B136" t="n">
+        <v>18930.939453125</v>
+      </c>
+      <c r="C136" t="n">
+        <v>1451258</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="1" t="n">
+        <v>41943</v>
+      </c>
+      <c r="B137" t="n">
+        <v>19075.529296875</v>
+      </c>
+      <c r="C137" t="n">
+        <v>1472311</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="1" t="n">
+        <v>41973</v>
+      </c>
+      <c r="B138" t="n">
+        <v>18789.01953125</v>
+      </c>
+      <c r="C138" t="n">
+        <v>1444579</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="1" t="n">
+        <v>42004</v>
+      </c>
+      <c r="B139" t="n">
+        <v>19893.30078125</v>
+      </c>
+      <c r="C139" t="n">
+        <v>1508392</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="1" t="n">
+        <v>42035</v>
+      </c>
+      <c r="B140" t="n">
+        <v>18812.330078125</v>
+      </c>
+      <c r="C140" t="n">
+        <v>1423196</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="1" t="n">
+        <v>42063</v>
+      </c>
+      <c r="B141" t="n">
+        <v>18772.26953125</v>
+      </c>
+      <c r="C141" t="n">
+        <v>1490792</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="1" t="n">
+        <v>42094</v>
+      </c>
+      <c r="B142" t="n">
+        <v>19508.41015625</v>
+      </c>
+      <c r="C142" t="n">
+        <v>1539313</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="1" t="n">
+        <v>42124</v>
+      </c>
+      <c r="B143" t="n">
+        <v>19340.98046875</v>
+      </c>
+      <c r="C143" t="n">
+        <v>1513581</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="1" t="n">
+        <v>42155</v>
+      </c>
+      <c r="B144" t="n">
+        <v>19231.6796875</v>
+      </c>
+      <c r="C144" t="n">
+        <v>1530988</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="1" t="n">
+        <v>42185</v>
+      </c>
+      <c r="B145" t="n">
+        <v>19301.900390625</v>
+      </c>
+      <c r="C145" t="n">
+        <v>1553760</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="1" t="n">
+        <v>42216</v>
+      </c>
+      <c r="B146" t="n">
+        <v>19932.05078125</v>
+      </c>
+      <c r="C146" t="n">
+        <v>1571146</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="1" t="n">
+        <v>42247</v>
+      </c>
+      <c r="B147" t="n">
+        <v>19601.869140625</v>
+      </c>
+      <c r="C147" t="n">
+        <v>1520245</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="1" t="n">
+        <v>42277</v>
+      </c>
+      <c r="B148" t="n">
+        <v>20045.330078125</v>
+      </c>
+      <c r="C148" t="n">
+        <v>1562475</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="1" t="n">
+        <v>42308</v>
+      </c>
+      <c r="B149" t="n">
+        <v>19896.400390625</v>
+      </c>
+      <c r="C149" t="n">
+        <v>1578120</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="1" t="n">
+        <v>42338</v>
+      </c>
+      <c r="B150" t="n">
+        <v>20120.26953125</v>
+      </c>
+      <c r="C150" t="n">
+        <v>1569766</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="1" t="n">
+        <v>42369</v>
+      </c>
+      <c r="B151" t="n">
+        <v>21370.580078125</v>
+      </c>
+      <c r="C151" t="n">
+        <v>1617107</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="1" t="n">
+        <v>42400</v>
+      </c>
+      <c r="B152" t="n">
+        <v>20194.390625</v>
+      </c>
+      <c r="C152" t="n">
+        <v>1501053</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="1" t="n">
+        <v>42429</v>
+      </c>
+      <c r="B153" t="n">
+        <v>20243.2109375</v>
+      </c>
+      <c r="C153" t="n">
+        <v>1605919</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="1" t="n">
+        <v>42460</v>
+      </c>
+      <c r="B154" t="n">
+        <v>20249.990234375</v>
+      </c>
+      <c r="C154" t="n">
+        <v>1671280</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="1" t="n">
+        <v>42490</v>
+      </c>
+      <c r="B155" t="n">
+        <v>20211.7890625</v>
+      </c>
+      <c r="C155" t="n">
+        <v>1646516</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="1" t="n">
+        <v>42521</v>
+      </c>
+      <c r="B156" t="n">
+        <v>20359.6796875</v>
+      </c>
+      <c r="C156" t="n">
+        <v>1679894</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="1" t="n">
+        <v>42551</v>
+      </c>
+      <c r="B157" t="n">
+        <v>20460.560546875</v>
+      </c>
+      <c r="C157" t="n">
+        <v>1643218</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="1" t="n">
+        <v>42582</v>
+      </c>
+      <c r="B158" t="n">
+        <v>20080.279296875</v>
+      </c>
+      <c r="C158" t="n">
+        <v>1668107</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="1" t="n">
+        <v>42613</v>
+      </c>
+      <c r="B159" t="n">
+        <v>20397.470703125</v>
+      </c>
+      <c r="C159" t="n">
+        <v>1683902</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="1" t="n">
+        <v>42643</v>
+      </c>
+      <c r="B160" t="n">
+        <v>20362.029296875</v>
+      </c>
+      <c r="C160" t="n">
+        <v>1684907</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="1" t="n">
+        <v>42674</v>
+      </c>
+      <c r="B161" t="n">
+        <v>20348.55078125</v>
+      </c>
+      <c r="C161" t="n">
+        <v>1685991</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="1" t="n">
+        <v>42704</v>
+      </c>
+      <c r="B162" t="n">
+        <v>20186.41015625</v>
+      </c>
+      <c r="C162" t="n">
+        <v>1695262</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="1" t="n">
+        <v>42735</v>
+      </c>
+      <c r="B163" t="n">
+        <v>21472.9296875</v>
+      </c>
+      <c r="C163" t="n">
+        <v>1725802</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="1" t="n">
+        <v>42766</v>
+      </c>
+      <c r="B164" t="n">
+        <v>20745.7109375</v>
+      </c>
+      <c r="C164" t="n">
+        <v>1624220</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="1" t="n">
+        <v>42794</v>
+      </c>
+      <c r="B165" t="n">
+        <v>20573.6796875</v>
+      </c>
+      <c r="C165" t="n">
+        <v>1682495</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="1" t="n">
+        <v>42825</v>
+      </c>
+      <c r="B166" t="n">
+        <v>21448.220703125</v>
+      </c>
+      <c r="C166" t="n">
+        <v>1727425</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="1" t="n">
+        <v>42855</v>
+      </c>
+      <c r="B167" t="n">
+        <v>20497.5390625</v>
+      </c>
+      <c r="C167" t="n">
+        <v>1716399</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="1" t="n">
+        <v>42886</v>
+      </c>
+      <c r="B168" t="n">
+        <v>20666.23046875</v>
+      </c>
+      <c r="C168" t="n">
+        <v>1793446</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="1" t="n">
+        <v>42916</v>
+      </c>
+      <c r="B169" t="n">
+        <v>20974.73046875</v>
+      </c>
+      <c r="C169" t="n">
+        <v>1774273</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="1" t="n">
+        <v>42947</v>
+      </c>
+      <c r="B170" t="n">
+        <v>20958.5</v>
+      </c>
+      <c r="C170" t="n">
+        <v>1779808</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="1" t="n">
+        <v>42978</v>
+      </c>
+      <c r="B171" t="n">
+        <v>20888.650390625</v>
+      </c>
+      <c r="C171" t="n">
+        <v>1786508</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="1" t="n">
+        <v>43008</v>
+      </c>
+      <c r="B172" t="n">
+        <v>21436.48046875</v>
+      </c>
+      <c r="C172" t="n">
+        <v>1775018</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="1" t="n">
+        <v>43039</v>
+      </c>
+      <c r="B173" t="n">
+        <v>21406.630859375</v>
+      </c>
+      <c r="C173" t="n">
+        <v>1807106</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="1" t="n">
+        <v>43069</v>
+      </c>
+      <c r="B174" t="n">
+        <v>21556.5</v>
+      </c>
+      <c r="C174" t="n">
+        <v>1804014</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="1" t="n">
+        <v>43100</v>
+      </c>
+      <c r="B175" t="n">
+        <v>22355.630859375</v>
+      </c>
+      <c r="C175" t="n">
+        <v>1837104</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="1" t="n">
+        <v>43131</v>
+      </c>
+      <c r="B176" t="n">
+        <v>22157.859375</v>
+      </c>
+      <c r="C176" t="n">
+        <v>1777342</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="1" t="n">
+        <v>43159</v>
+      </c>
+      <c r="B177" t="n">
+        <v>21732.689453125</v>
+      </c>
+      <c r="C177" t="n">
+        <v>1807468</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="1" t="n">
+        <v>43190</v>
+      </c>
+      <c r="B178" t="n">
+        <v>22385.140625</v>
+      </c>
+      <c r="C178" t="n">
+        <v>1860698</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="1" t="n">
+        <v>43220</v>
+      </c>
+      <c r="B179" t="n">
+        <v>22098.220703125</v>
+      </c>
+      <c r="C179" t="n">
+        <v>1830789</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="1" t="n">
+        <v>43251</v>
+      </c>
+      <c r="B180" t="n">
+        <v>22404.859375</v>
+      </c>
+      <c r="C180" t="n">
+        <v>1890857</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="1" t="n">
+        <v>43281</v>
+      </c>
+      <c r="B181" t="n">
+        <v>22203.880859375</v>
+      </c>
+      <c r="C181" t="n">
+        <v>1813834</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="1" t="n">
+        <v>43312</v>
+      </c>
+      <c r="B182" t="n">
+        <v>22751.119140625</v>
+      </c>
+      <c r="C182" t="n">
+        <v>1894599</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="1" t="n">
+        <v>43343</v>
+      </c>
+      <c r="B183" t="n">
+        <v>22543.369140625</v>
+      </c>
+      <c r="C183" t="n">
+        <v>1888021</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="1" t="n">
+        <v>43373</v>
+      </c>
+      <c r="B184" t="n">
+        <v>22496.490234375</v>
+      </c>
+      <c r="C184" t="n">
+        <v>1857705</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="1" t="n">
+        <v>43404</v>
+      </c>
+      <c r="B185" t="n">
+        <v>22681.169921875</v>
+      </c>
+      <c r="C185" t="n">
+        <v>1922130</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="1" t="n">
+        <v>43434</v>
+      </c>
+      <c r="B186" t="n">
+        <v>22436.900390625</v>
+      </c>
+      <c r="C186" t="n">
+        <v>1902380</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="1" t="n">
+        <v>43465</v>
+      </c>
+      <c r="B187" t="n">
+        <v>23772.9296875</v>
+      </c>
+      <c r="C187" t="n">
+        <v>1935968</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="1" t="n">
+        <v>43496</v>
+      </c>
+      <c r="B188" t="n">
+        <v>22738.30078125</v>
+      </c>
+      <c r="C188" t="n">
+        <v>1872444</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="1" t="n">
+        <v>43524</v>
+      </c>
+      <c r="B189" t="n">
+        <v>22215.599609375</v>
+      </c>
+      <c r="C189" t="n">
+        <v>1914717</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="1" t="n">
+        <v>43555</v>
+      </c>
+      <c r="B190" t="n">
+        <v>22811.759765625</v>
+      </c>
+      <c r="C190" t="n">
+        <v>1969696</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="1" t="n">
+        <v>43585</v>
+      </c>
+      <c r="B191" t="n">
+        <v>22564.490234375</v>
+      </c>
+      <c r="C191" t="n">
+        <v>1962253</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="1" t="n">
+        <v>43616</v>
+      </c>
+      <c r="B192" t="n">
+        <v>23959.439453125</v>
+      </c>
+      <c r="C192" t="n">
+        <v>1931882</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="1" t="n">
+        <v>43646</v>
+      </c>
+      <c r="B193" t="n">
+        <v>23806.099609375</v>
+      </c>
+      <c r="C193" t="n">
+        <v>1885197</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="1" t="n">
+        <v>43677</v>
+      </c>
+      <c r="B194" t="n">
+        <v>23839.30078125</v>
+      </c>
+      <c r="C194" t="n">
+        <v>1939817</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="1" t="n">
+        <v>43708</v>
+      </c>
+      <c r="B195" t="n">
+        <v>23658.130859375</v>
+      </c>
+      <c r="C195" t="n">
+        <v>1917355</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="1" t="n">
+        <v>43738</v>
+      </c>
+      <c r="B196" t="n">
+        <v>24165.1796875</v>
+      </c>
+      <c r="C196" t="n">
+        <v>1924512</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="1" t="n">
+        <v>43769</v>
+      </c>
+      <c r="B197" t="n">
+        <v>24530.16015625</v>
+      </c>
+      <c r="C197" t="n">
+        <v>1959668</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="1" t="n">
+        <v>43799</v>
+      </c>
+      <c r="B198" t="n">
+        <v>23898.529296875</v>
+      </c>
+      <c r="C198" t="n">
+        <v>1910515</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="1" t="n">
+        <v>43830</v>
+      </c>
+      <c r="B199" t="n">
+        <v>27018.470703125</v>
+      </c>
+      <c r="C199" t="n">
+        <v>1924919</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="1" t="n">
+        <v>43861</v>
+      </c>
+      <c r="B200" t="n">
+        <v>25826.4609375</v>
+      </c>
+      <c r="C200" t="n">
+        <v>1861696</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="1" t="n">
+        <v>43890</v>
+      </c>
+      <c r="B201" t="n">
+        <v>25609.560546875</v>
+      </c>
+      <c r="C201" t="n">
+        <v>1903195</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="1" t="n">
+        <v>43921</v>
+      </c>
+      <c r="B202" t="n">
+        <v>25611.650390625</v>
+      </c>
+      <c r="C202" t="n">
+        <v>1962593</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="1" t="n">
+        <v>43951</v>
+      </c>
+      <c r="B203" t="n">
+        <v>26372.369140625</v>
+      </c>
+      <c r="C203" t="n">
+        <v>1569809</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="1" t="n">
+        <v>43982</v>
+      </c>
+      <c r="B204" t="n">
+        <v>28120.939453125</v>
+      </c>
+      <c r="C204" t="n">
+        <v>1460091</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="1" t="n">
+        <v>44012</v>
+      </c>
+      <c r="B205" t="n">
+        <v>26703.55078125</v>
+      </c>
+      <c r="C205" t="n">
+        <v>1397937</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="1" t="n">
+        <v>44043</v>
+      </c>
+      <c r="B206" t="n">
+        <v>26135.630859375</v>
+      </c>
+      <c r="C206" t="n">
+        <v>1597113</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="1" t="n">
+        <v>44074</v>
+      </c>
+      <c r="B207" t="n">
+        <v>25878.669921875</v>
+      </c>
+      <c r="C207" t="n">
+        <v>1624478</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="1" t="n">
+        <v>44104</v>
+      </c>
+      <c r="B208" t="n">
+        <v>25852.01953125</v>
+      </c>
+      <c r="C208" t="n">
+        <v>1653032</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="1" t="n">
+        <v>44135</v>
+      </c>
+      <c r="B209" t="n">
+        <v>25828.41015625</v>
+      </c>
+      <c r="C209" t="n">
+        <v>1674668</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="1" t="n">
+        <v>44165</v>
+      </c>
+      <c r="B210" t="n">
+        <v>25905.830078125</v>
+      </c>
+      <c r="C210" t="n">
+        <v>1658616</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="1" t="n">
+        <v>44196</v>
+      </c>
+      <c r="B211" t="n">
+        <v>26362.7109375</v>
+      </c>
+      <c r="C211" t="n">
+        <v>1747440</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="1" t="n">
+        <v>44227</v>
+      </c>
+      <c r="B212" t="n">
+        <v>26257.8203125</v>
+      </c>
+      <c r="C212" t="n">
+        <v>1652224</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="1" t="n">
+        <v>44255</v>
+      </c>
+      <c r="B213" t="n">
+        <v>26059.05078125</v>
+      </c>
+      <c r="C213" t="n">
+        <v>1756519</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="1" t="n">
+        <v>44286</v>
+      </c>
+      <c r="B214" t="n">
+        <v>27364.029296875</v>
+      </c>
+      <c r="C214" t="n">
+        <v>1803984</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="1" t="n">
+        <v>44316</v>
+      </c>
+      <c r="B215" t="n">
+        <v>26667.630859375</v>
+      </c>
+      <c r="C215" t="n">
+        <v>1740784</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="1" t="n">
+        <v>44347</v>
+      </c>
+      <c r="B216" t="n">
+        <v>26777.76953125</v>
+      </c>
+      <c r="C216" t="n">
+        <v>1803412</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="1" t="n">
+        <v>44377</v>
+      </c>
+      <c r="B217" t="n">
+        <v>26312.55078125</v>
+      </c>
+      <c r="C217" t="n">
+        <v>1831156</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="1" t="n">
+        <v>44408</v>
+      </c>
+      <c r="B218" t="n">
+        <v>27005.400390625</v>
+      </c>
+      <c r="C218" t="n">
+        <v>1866512</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="1" t="n">
+        <v>44439</v>
+      </c>
+      <c r="B219" t="n">
+        <v>27988.060546875</v>
+      </c>
+      <c r="C219" t="n">
+        <v>1872658</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="1" t="n">
+        <v>44469</v>
+      </c>
+      <c r="B220" t="n">
+        <v>27847.69921875</v>
+      </c>
+      <c r="C220" t="n">
+        <v>1879053</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="1" t="n">
+        <v>44500</v>
+      </c>
+      <c r="B221" t="n">
+        <v>28020.4296875</v>
+      </c>
+      <c r="C221" t="n">
+        <v>1913789</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="1" t="n">
+        <v>44530</v>
+      </c>
+      <c r="B222" t="n">
+        <v>28049.9296875</v>
+      </c>
+      <c r="C222" t="n">
+        <v>1939371</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="1" t="n">
+        <v>44561</v>
+      </c>
+      <c r="B223" t="n">
+        <v>29547.439453125</v>
+      </c>
+      <c r="C223" t="n">
+        <v>1972032</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="1" t="n">
+        <v>44592</v>
+      </c>
+      <c r="B224" t="n">
+        <v>28563.509765625</v>
+      </c>
+      <c r="C224" t="n">
+        <v>1864996</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="1" t="n">
+        <v>44620</v>
+      </c>
+      <c r="B225" t="n">
+        <v>28044.1796875</v>
+      </c>
+      <c r="C225" t="n">
+        <v>1956958</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="1" t="n">
+        <v>44651</v>
+      </c>
+      <c r="B226" t="n">
+        <v>29497.359375</v>
+      </c>
+      <c r="C226" t="n">
+        <v>2031036</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="1" t="n">
+        <v>44681</v>
+      </c>
+      <c r="B227" t="n">
+        <v>28757.5</v>
+      </c>
+      <c r="C227" t="n">
+        <v>1977626</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="1" t="n">
+        <v>44712</v>
+      </c>
+      <c r="B228" t="n">
+        <v>29622.970703125</v>
+      </c>
+      <c r="C228" t="n">
+        <v>2038706</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="1" t="n">
+        <v>44742</v>
+      </c>
+      <c r="B229" t="n">
+        <v>28993.16015625</v>
+      </c>
+      <c r="C229" t="n">
+        <v>2018402</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="1" t="n">
+        <v>44773</v>
+      </c>
+      <c r="B230" t="n">
+        <v>29888.73046875</v>
+      </c>
+      <c r="C230" t="n">
+        <v>2054737</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="1" t="n">
+        <v>44804</v>
+      </c>
+      <c r="B231" t="n">
+        <v>29965.650390625</v>
+      </c>
+      <c r="C231" t="n">
+        <v>2077092</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="1" t="n">
+        <v>44834</v>
+      </c>
+      <c r="B232" t="n">
+        <v>29790.119140625</v>
+      </c>
+      <c r="C232" t="n">
+        <v>2044732</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="1" t="n">
+        <v>44865</v>
+      </c>
+      <c r="B233" t="n">
+        <v>29994.880859375</v>
+      </c>
+      <c r="C233" t="n">
+        <v>1985841</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="1" t="n">
+        <v>44895</v>
+      </c>
+      <c r="B234" t="n">
+        <v>29607.4296875</v>
+      </c>
+      <c r="C234" t="n">
+        <v>1996282</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="1" t="n">
+        <v>44926</v>
+      </c>
+      <c r="B235" t="n">
+        <v>30054.5</v>
+      </c>
+      <c r="C235" t="n">
+        <v>2020997</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="1" t="n">
+        <v>44957</v>
+      </c>
+      <c r="B236" t="n">
+        <v>30440.259765625</v>
+      </c>
+      <c r="C236" t="n">
+        <v>2020338</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="1" t="n">
+        <v>44985</v>
+      </c>
+      <c r="B237" t="n">
+        <v>29792.869140625</v>
+      </c>
+      <c r="C237" t="n">
+        <v>2105974</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="1" t="n">
+        <v>45016</v>
+      </c>
+      <c r="B238" t="n">
+        <v>31154.310546875</v>
+      </c>
+      <c r="C238" t="n">
+        <v>2159049</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="1" t="n">
+        <v>45046</v>
+      </c>
+      <c r="B239" t="n">
+        <v>30464.609375</v>
+      </c>
+      <c r="C239" t="n">
+        <v>2071926</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="1" t="n">
+        <v>45077</v>
+      </c>
+      <c r="B240" t="n">
+        <v>32248.720703125</v>
+      </c>
+      <c r="C240" t="n">
+        <v>2138001</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="1" t="n">
+        <v>45107</v>
+      </c>
+      <c r="B241" t="n">
+        <v>31695.740234375</v>
+      </c>
+      <c r="C241" t="n">
+        <v>2099920</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="1" t="n">
+        <v>45138</v>
+      </c>
+      <c r="B242" t="n">
+        <v>33184.578125</v>
+      </c>
+      <c r="C242" t="n">
+        <v>2107284</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="1" t="n">
+        <v>45169</v>
+      </c>
+      <c r="B243" t="n">
+        <v>32704.9296875</v>
+      </c>
+      <c r="C243" t="n">
+        <v>2094278</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="1" t="n">
+        <v>45199</v>
+      </c>
+      <c r="B244" t="n">
+        <v>33114.21875</v>
+      </c>
+      <c r="C244" t="n">
+        <v>2103843</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="1" t="n">
+        <v>45230</v>
+      </c>
+      <c r="B245" t="n">
+        <v>33275.75</v>
+      </c>
+      <c r="C245" t="n">
+        <v>2133925</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="1" t="n">
+        <v>45260</v>
+      </c>
+      <c r="B246" t="n">
+        <v>33329.828125</v>
+      </c>
+      <c r="C246" t="n">
+        <v>2105433</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="1" t="n">
+        <v>45291</v>
+      </c>
+      <c r="B247" t="n">
+        <v>34159.8984375</v>
+      </c>
+      <c r="C247" t="n">
+        <v>2138144</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="1" t="n">
+        <v>45322</v>
+      </c>
+      <c r="B248" t="n">
+        <v>33880.3515625</v>
+      </c>
+      <c r="C248" t="n">
+        <v>2093134</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="1" t="n">
+        <v>45351</v>
+      </c>
+      <c r="B249" t="n">
+        <v>33285.8203125</v>
+      </c>
+      <c r="C249" t="n">
+        <v>2138524</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="1" t="n">
+        <v>45382</v>
+      </c>
+      <c r="B250" t="n">
+        <v>34355.55859375</v>
+      </c>
+      <c r="C250" t="n">
+        <v>2158279</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="1" t="n">
+        <v>45412</v>
+      </c>
+      <c r="B251" t="n">
+        <v>34291.9296875</v>
+      </c>
+      <c r="C251" t="n">
+        <v>2128643</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="1" t="n">
+        <v>45443</v>
+      </c>
+      <c r="B252" t="n">
+        <v>34827.9609375</v>
+      </c>
+      <c r="C252" t="n">
+        <v>2176498</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="1" t="n">
+        <v>45473</v>
+      </c>
+      <c r="B253" t="n">
+        <v>34632.37890625</v>
+      </c>
+      <c r="C253" t="n">
+        <v>2146387</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="1" t="n">
+        <v>45504</v>
+      </c>
+      <c r="B254" t="n">
+        <v>35385.1015625</v>
+      </c>
+      <c r="C254" t="n">
+        <v>2184125</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="1" t="n">
+        <v>45535</v>
+      </c>
+      <c r="B255" t="n">
+        <v>35193.578125</v>
+      </c>
+      <c r="C255" t="n">
+        <v>2144976</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="1" t="n">
+        <v>45565</v>
+      </c>
+      <c r="B256" t="n">
+        <v>35375.8984375</v>
+      </c>
+      <c r="C256" t="n">
+        <v>2160783</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="1" t="n">
+        <v>45596</v>
+      </c>
+      <c r="B257" t="n">
+        <v>35588.25</v>
+      </c>
+      <c r="C257" t="n">
+        <v>2206846</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="1" t="n">
+        <v>45626</v>
+      </c>
+      <c r="B258" t="n">
+        <v>35348.12890625</v>
+      </c>
+      <c r="C258" t="n">
+        <v>2157762</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="1" t="n">
+        <v>45657</v>
+      </c>
+      <c r="B259" t="n">
+        <v>36905.26953125</v>
+      </c>
+      <c r="C259" t="n">
+        <v>2219499</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="1" t="n">
+        <v>45688</v>
+      </c>
+      <c r="B260" t="n">
+        <v>35750.5390625</v>
+      </c>
+      <c r="C260" t="n">
+        <v>2123418</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="1" t="n">
+        <v>45716</v>
+      </c>
+      <c r="B261" t="n">
+        <v>35698.19921875</v>
+      </c>
+      <c r="C261" t="n">
+        <v>2158065</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="1" t="n">
+        <v>45747</v>
+      </c>
+      <c r="B262" t="n">
+        <v>36120.87890625</v>
+      </c>
+      <c r="C262" t="n">
+        <v>2230869</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="1" t="n">
+        <v>45777</v>
+      </c>
+      <c r="B263" t="n">
+        <v>35102.921875</v>
+      </c>
+      <c r="C263" t="n">
+        <v>2226931</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="1" t="n">
+        <v>45808</v>
+      </c>
+      <c r="B264" t="n">
+        <v>36328.25</v>
+      </c>
+      <c r="C264" t="n">
+        <v>2242332</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="1" t="n">
+        <v>45838</v>
+      </c>
+      <c r="B265" t="n">
+        <v>36419.63062428</v>
+      </c>
+      <c r="C265" t="n">
+        <v>2226937</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="1" t="n">
+        <v>45869</v>
+      </c>
+      <c r="B266" t="n">
+        <v>36635.05495667</v>
+      </c>
+      <c r="C266" t="n">
+        <v>2260926</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="1" t="n">
+        <v>45900</v>
+      </c>
+      <c r="B267" t="n">
+        <v>37422.94386606</v>
+      </c>
+      <c r="C267" t="n">
+        <v>2192103</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="1" t="n">
+        <v>45930</v>
+      </c>
+      <c r="B268" t="n">
+        <v>37122.61066755</v>
+      </c>
+      <c r="C268" t="n">
+        <v>2255383</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="1" t="n">
+        <v>45961</v>
+      </c>
+      <c r="B269" t="n">
+        <v>36931.49068016</v>
+      </c>
+      <c r="C269" t="n">
+        <v>2281237</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="1" t="n">
+        <v>45991</v>
+      </c>
+      <c r="B270" t="n">
+        <v>37448.0298499</v>
+      </c>
+      <c r="C270" t="n">
+        <v>2243854</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="1" t="n">
+        <v>46022</v>
+      </c>
+      <c r="B271" t="n">
+        <v>37201.39659823</v>
+      </c>
+      <c r="C271" t="n">
+        <v>2308549</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="1" t="n">
+        <v>46053</v>
+      </c>
+      <c r="B272" t="n">
+        <v>37576.78317798</v>
+      </c>
+      <c r="C272" t="n">
+        <v>2181704</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="1" t="n">
+        <v>46081</v>
+      </c>
+      <c r="B273" t="n">
+        <v>37780.78510248</v>
+      </c>
+      <c r="C273" t="n">
+        <v>2272743</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="1" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B274" t="n">
+        <v>38092.43616123</v>
+      </c>
+      <c r="C274" t="n">
+        <v>2325278</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="1" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B275" t="n">
+        <v>38216.971436</v>
+      </c>
+      <c r="C275" t="n">
+        <v>2256214</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="1" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B276" t="n">
+        <v>39021.55552756</v>
+      </c>
+      <c r="C276" t="n">
+        <v>2306128</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>